<commit_message>
Record 1000-run robustness results
</commit_message>
<xml_diff>
--- a/test-results-team6/test-robustness-team6.xlsx
+++ b/test-results-team6/test-robustness-team6.xlsx
@@ -525,7 +525,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Team 6 measured runs (current source)</t>
+          <t>Team 6 measured runs (2026-10-27)</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>100/100 completed cleanly</t>
+          <t>1000/1000 completed cleanly (input: no_conflict_2Txs.txt)</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>100/100 completed cleanly</t>
+          <t>1000/1000 completed cleanly</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>100/100 completed cleanly</t>
+          <t>1000/1000 completed cleanly</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>100/100 completed cleanly</t>
+          <t>1000/1000 completed cleanly</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>100/100 completed cleanly</t>
+          <t>1000/1000 completed cleanly</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>100/100 completed cleanly</t>
+          <t>1000/1000 completed cleanly</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>100/100 completed cleanly</t>
+          <t>1000/1000 completed cleanly</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>100/100 completed cleanly</t>
+          <t>1000/1000 completed cleanly</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>100/100 completed cleanly</t>
+          <t>1000/1000 completed cleanly</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>100/100 completed cleanly</t>
+          <t>1000/1000 completed cleanly</t>
         </is>
       </c>
     </row>

</xml_diff>